<commit_message>
fix: tabtools 2.5.6 puttab panel headings unmerged and sized into column B
puttab panel() heading rows (and so stacktab panel headings) are no
longer merged across the table. The heading sits in the row-label column,
bold and ruled above, with the other cells blank, and its text now counts
toward that column's width (up to the 50-character cap); before, headings
were excluded from the width. puttab.sthlp and the README changelog are
updated and every file moves to 2.5.6.

QA: the panel merge assertions in test_puttab_v230, test_puttab_v240 and
test_stacktab_v230 now assert no merge, and test_puttab_v230 adds a
regression block for unmerged headings and heading-driven column width.
The demo workbooks are regenerated: demo_puttab and demo_stacktab for
this change, and demo_crosstab, demo_desctab and demo_table1, which still
carried the footnote wording from before 2.5.5.
</commit_message>
<xml_diff>
--- a/tabtools/demo/demo_puttab.xlsx
+++ b/tabtools/demo/demo_puttab.xlsx
@@ -1472,7 +1472,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="1.7109375" style="1" customWidth="true"/>
-    <col min="2" max="2" width="16.7109375" style="1" customWidth="true"/>
+    <col min="2" max="2" width="21.7109375" style="1" customWidth="true"/>
     <col min="3" max="3" width="10.7109375" style="1" customWidth="true"/>
     <col min="4" max="4" width="14.7109375" style="1" customWidth="true"/>
   </cols>
@@ -1618,10 +1618,8 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B6:D6"/>
     <mergeCell ref="B9:D9"/>
     <mergeCell ref="B10:D10"/>
   </mergeCells>

</xml_diff>